<commit_message>
Fake employee list: Team One/Two/Three and a Shufflers team
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0138Z6CMxeV6Xe9DnVMeD824
</commit_message>
<xml_diff>
--- a/demo/PTF-fake-employees-200.xlsx
+++ b/demo/PTF-fake-employees-200.xlsx
@@ -560,7 +560,7 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -767,7 +767,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -809,7 +809,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -937,7 +937,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -979,7 +979,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1062,7 +1062,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1186,7 +1186,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1311,7 +1311,7 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -1477,7 +1477,7 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1560,7 +1560,7 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -1643,7 +1643,7 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -1726,7 +1726,7 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1771,7 +1771,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -1809,7 +1809,7 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -1888,7 +1888,7 @@
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -1967,7 +1967,7 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2012,7 +2012,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -2050,7 +2050,7 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2133,7 @@
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2299,7 +2299,7 @@
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2465,7 +2465,7 @@
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2510,7 +2510,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -2552,7 +2552,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2635,7 +2635,7 @@
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -2714,7 +2714,7 @@
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -2797,7 +2797,7 @@
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -2880,7 +2880,7 @@
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2963,7 +2963,7 @@
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3125,7 +3125,7 @@
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3295,7 +3295,7 @@
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3340,7 +3340,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -3382,7 +3382,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3465,7 +3465,7 @@
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -3544,7 +3544,7 @@
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3585,7 +3585,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -3627,7 +3627,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3710,7 +3710,7 @@
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3751,7 +3751,7 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -3789,7 +3789,7 @@
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3872,7 +3872,7 @@
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3955,7 +3955,7 @@
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3996,7 +3996,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -4034,7 +4034,7 @@
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4117,7 +4117,7 @@
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4162,7 +4162,7 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -4200,7 +4200,7 @@
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4241,7 +4241,7 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -4279,7 +4279,7 @@
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -4324,7 +4324,7 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -4362,7 +4362,7 @@
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -4445,7 +4445,7 @@
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -4565,7 +4565,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -4603,7 +4603,7 @@
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4644,7 +4644,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -4682,7 +4682,7 @@
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4727,7 +4727,7 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -4765,7 +4765,7 @@
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -4810,7 +4810,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -4848,7 +4848,7 @@
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -4893,7 +4893,7 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -4931,7 +4931,7 @@
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -5018,7 +5018,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -5101,7 +5101,7 @@
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -5184,7 +5184,7 @@
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -5225,7 +5225,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -5267,7 +5267,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -5354,7 +5354,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -5437,7 +5437,7 @@
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -5524,7 +5524,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -5607,7 +5607,7 @@
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -5690,7 +5690,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -5777,7 +5777,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -5822,7 +5822,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -5864,7 +5864,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -5909,7 +5909,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -5947,7 +5947,7 @@
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -6034,7 +6034,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -6117,7 +6117,7 @@
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -6158,7 +6158,7 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -6196,7 +6196,7 @@
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -6279,7 +6279,7 @@
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -6320,7 +6320,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -6362,7 +6362,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -6445,7 +6445,7 @@
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -6528,7 +6528,7 @@
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -6569,7 +6569,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -6611,7 +6611,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -6694,7 +6694,7 @@
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -6739,7 +6739,7 @@
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -6781,7 +6781,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -6826,7 +6826,7 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -6864,7 +6864,7 @@
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -6905,7 +6905,7 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -6943,7 +6943,7 @@
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -7026,7 +7026,7 @@
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -7113,7 +7113,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -7158,7 +7158,7 @@
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -7283,7 +7283,7 @@
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -7328,7 +7328,7 @@
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -7370,7 +7370,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -7453,7 +7453,7 @@
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -7536,7 +7536,7 @@
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -7577,7 +7577,7 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -7615,7 +7615,7 @@
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -7698,7 +7698,7 @@
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -7785,7 +7785,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -7830,7 +7830,7 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -7955,7 +7955,7 @@
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -7996,7 +7996,7 @@
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -8034,7 +8034,7 @@
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -8079,7 +8079,7 @@
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -8121,7 +8121,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -8166,7 +8166,7 @@
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -8204,7 +8204,7 @@
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -8249,7 +8249,7 @@
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -8287,7 +8287,7 @@
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -8332,7 +8332,7 @@
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -8370,7 +8370,7 @@
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -8453,7 +8453,7 @@
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -8540,7 +8540,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -8585,7 +8585,7 @@
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -8623,7 +8623,7 @@
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -8702,7 +8702,7 @@
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -8743,7 +8743,7 @@
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -8785,7 +8785,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -8868,7 +8868,7 @@
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -8909,7 +8909,7 @@
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -8947,7 +8947,7 @@
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -9030,7 +9030,7 @@
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -9071,7 +9071,7 @@
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -9113,7 +9113,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -9196,7 +9196,7 @@
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -9237,7 +9237,7 @@
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -9275,7 +9275,7 @@
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -9320,7 +9320,7 @@
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -9358,7 +9358,7 @@
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -9403,7 +9403,7 @@
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -9445,7 +9445,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -9490,7 +9490,7 @@
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -9528,7 +9528,7 @@
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -9615,7 +9615,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -9698,7 +9698,7 @@
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -9739,7 +9739,7 @@
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -9781,7 +9781,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -9864,7 +9864,7 @@
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -9909,7 +9909,7 @@
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -9947,7 +9947,7 @@
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -9992,7 +9992,7 @@
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -10030,7 +10030,7 @@
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -10117,7 +10117,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -10162,7 +10162,7 @@
       </c>
       <c r="Q117" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -10204,7 +10204,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -10287,7 +10287,7 @@
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -10374,7 +10374,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -10461,7 +10461,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -10548,7 +10548,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -10593,7 +10593,7 @@
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -10631,7 +10631,7 @@
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -10676,7 +10676,7 @@
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -10714,7 +10714,7 @@
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -10755,7 +10755,7 @@
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -10797,7 +10797,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -10880,7 +10880,7 @@
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -10921,7 +10921,7 @@
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -10963,7 +10963,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -11008,7 +11008,7 @@
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -11046,7 +11046,7 @@
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -11091,7 +11091,7 @@
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -11133,7 +11133,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -11178,7 +11178,7 @@
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -11216,7 +11216,7 @@
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -11257,7 +11257,7 @@
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -11299,7 +11299,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -11382,7 +11382,7 @@
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -11469,7 +11469,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -11556,7 +11556,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -11601,7 +11601,7 @@
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -11639,7 +11639,7 @@
       <c r="G135" t="inlineStr"/>
       <c r="H135" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -11722,7 +11722,7 @@
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -11767,7 +11767,7 @@
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -11805,7 +11805,7 @@
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -11888,7 +11888,7 @@
       <c r="G138" t="inlineStr"/>
       <c r="H138" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -11933,7 +11933,7 @@
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -11971,7 +11971,7 @@
       <c r="G139" t="inlineStr"/>
       <c r="H139" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -12012,7 +12012,7 @@
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -12050,7 +12050,7 @@
       <c r="G140" t="inlineStr"/>
       <c r="H140" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -12133,7 +12133,7 @@
       <c r="G141" t="inlineStr"/>
       <c r="H141" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -12178,7 +12178,7 @@
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -12216,7 +12216,7 @@
       <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -12257,7 +12257,7 @@
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -12299,7 +12299,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -12344,7 +12344,7 @@
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -12382,7 +12382,7 @@
       <c r="G144" t="inlineStr"/>
       <c r="H144" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -12423,7 +12423,7 @@
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -12461,7 +12461,7 @@
       <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -12544,7 +12544,7 @@
       <c r="G146" t="inlineStr"/>
       <c r="H146" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -12589,7 +12589,7 @@
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -12627,7 +12627,7 @@
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -12710,7 +12710,7 @@
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -12755,7 +12755,7 @@
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -12793,7 +12793,7 @@
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -12838,7 +12838,7 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -12880,7 +12880,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -12963,7 +12963,7 @@
       <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -13008,7 +13008,7 @@
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -13050,7 +13050,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -13137,7 +13137,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -13220,7 +13220,7 @@
       <c r="G154" t="inlineStr"/>
       <c r="H154" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -13265,7 +13265,7 @@
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -13303,7 +13303,7 @@
       <c r="G155" t="inlineStr"/>
       <c r="H155" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -13386,7 +13386,7 @@
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -13427,7 +13427,7 @@
       </c>
       <c r="Q156" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -13465,7 +13465,7 @@
       <c r="G157" t="inlineStr"/>
       <c r="H157" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -13506,7 +13506,7 @@
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -13544,7 +13544,7 @@
       <c r="G158" t="inlineStr"/>
       <c r="H158" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -13585,7 +13585,7 @@
       </c>
       <c r="Q158" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -13627,7 +13627,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -13672,7 +13672,7 @@
       </c>
       <c r="Q159" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -13710,7 +13710,7 @@
       <c r="G160" t="inlineStr"/>
       <c r="H160" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -13751,7 +13751,7 @@
       </c>
       <c r="Q160" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -13789,7 +13789,7 @@
       <c r="G161" t="inlineStr"/>
       <c r="H161" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -13834,7 +13834,7 @@
       </c>
       <c r="Q161" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -13872,7 +13872,7 @@
       <c r="G162" t="inlineStr"/>
       <c r="H162" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -13955,7 +13955,7 @@
       <c r="G163" t="inlineStr"/>
       <c r="H163" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -14000,7 +14000,7 @@
       </c>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -14038,7 +14038,7 @@
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -14121,7 +14121,7 @@
       <c r="G165" t="inlineStr"/>
       <c r="H165" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -14162,7 +14162,7 @@
       </c>
       <c r="Q165" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -14204,7 +14204,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -14249,7 +14249,7 @@
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -14287,7 +14287,7 @@
       <c r="G167" t="inlineStr"/>
       <c r="H167" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -14332,7 +14332,7 @@
       </c>
       <c r="Q167" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -14370,7 +14370,7 @@
       <c r="G168" t="inlineStr"/>
       <c r="H168" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -14453,7 +14453,7 @@
       <c r="G169" t="inlineStr"/>
       <c r="H169" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -14494,7 +14494,7 @@
       </c>
       <c r="Q169" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -14536,7 +14536,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -14619,7 +14619,7 @@
       <c r="G171" t="inlineStr"/>
       <c r="H171" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -14664,7 +14664,7 @@
       </c>
       <c r="Q171" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -14706,7 +14706,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -14789,7 +14789,7 @@
       <c r="G173" t="inlineStr"/>
       <c r="H173" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -14830,7 +14830,7 @@
       </c>
       <c r="Q173" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -14872,7 +14872,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -14959,7 +14959,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -15042,7 +15042,7 @@
       <c r="G176" t="inlineStr"/>
       <c r="H176" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -15083,7 +15083,7 @@
       </c>
       <c r="Q176" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -15125,7 +15125,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -15170,7 +15170,7 @@
       </c>
       <c r="Q177" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -15212,7 +15212,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -15257,7 +15257,7 @@
       </c>
       <c r="Q178" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -15295,7 +15295,7 @@
       <c r="G179" t="inlineStr"/>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -15378,7 +15378,7 @@
       <c r="G180" t="inlineStr"/>
       <c r="H180" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -15419,7 +15419,7 @@
       </c>
       <c r="Q180" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -15457,7 +15457,7 @@
       <c r="G181" t="inlineStr"/>
       <c r="H181" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -15540,7 +15540,7 @@
       <c r="G182" t="inlineStr"/>
       <c r="H182" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -15623,7 +15623,7 @@
       <c r="G183" t="inlineStr"/>
       <c r="H183" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -15706,7 +15706,7 @@
       <c r="G184" t="inlineStr"/>
       <c r="H184" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -15789,7 +15789,7 @@
       <c r="G185" t="inlineStr"/>
       <c r="H185" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -15876,7 +15876,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -15921,7 +15921,7 @@
       </c>
       <c r="Q186" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -15963,7 +15963,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -16008,7 +16008,7 @@
       </c>
       <c r="Q187" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -16046,7 +16046,7 @@
       <c r="G188" t="inlineStr"/>
       <c r="H188" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -16087,7 +16087,7 @@
       </c>
       <c r="Q188" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -16125,7 +16125,7 @@
       <c r="G189" t="inlineStr"/>
       <c r="H189" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -16208,7 +16208,7 @@
       <c r="G190" t="inlineStr"/>
       <c r="H190" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -16249,7 +16249,7 @@
       </c>
       <c r="Q190" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -16287,7 +16287,7 @@
       <c r="G191" t="inlineStr"/>
       <c r="H191" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -16332,7 +16332,7 @@
       </c>
       <c r="Q191" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -16370,7 +16370,7 @@
       <c r="G192" t="inlineStr"/>
       <c r="H192" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -16457,7 +16457,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -16502,7 +16502,7 @@
       </c>
       <c r="Q193" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -16540,7 +16540,7 @@
       <c r="G194" t="inlineStr"/>
       <c r="H194" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -16581,7 +16581,7 @@
       </c>
       <c r="Q194" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -16619,7 +16619,7 @@
       <c r="G195" t="inlineStr"/>
       <c r="H195" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -16664,7 +16664,7 @@
       </c>
       <c r="Q195" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -16706,7 +16706,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -16751,7 +16751,7 @@
       </c>
       <c r="Q196" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -16789,7 +16789,7 @@
       <c r="G197" t="inlineStr"/>
       <c r="H197" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Shufflers</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -16830,7 +16830,7 @@
       </c>
       <c r="Q197" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -16868,7 +16868,7 @@
       <c r="G198" t="inlineStr"/>
       <c r="H198" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -16951,7 +16951,7 @@
       <c r="G199" t="inlineStr"/>
       <c r="H199" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team One</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -16996,7 +16996,7 @@
       </c>
       <c r="Q199" t="inlineStr">
         <is>
-          <t>Luka Chkheidze</t>
+          <t>Mariami Beridze</t>
         </is>
       </c>
     </row>
@@ -17034,7 +17034,7 @@
       <c r="G200" t="inlineStr"/>
       <c r="H200" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Team Two</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -17079,7 +17079,7 @@
       </c>
       <c r="Q200" t="inlineStr">
         <is>
-          <t>Mariami Beridze</t>
+          <t>Luka Chkheidze</t>
         </is>
       </c>
     </row>
@@ -17117,7 +17117,7 @@
       <c r="G201" t="inlineStr"/>
       <c r="H201" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Team Three</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">

</xml_diff>